<commit_message>
fix: harden HTML extraction after live checks on all 20 homepage sources
- Skip hidden headings (Jago News has a hidden <h1> in every card)
- Strip <time>/date/tag labels, also inside headings
- Fall back to the card's single heading for empty overlay links
  (Bhorer Kagoj, RTV, BSS, Dhaka Times)
- Daily Star Bangla: match any /news-NNNN path (21 -> 100 headlines)
- Tests for the new cases; spreadsheet updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GQT3E1BZYoenUycoK4dun1
</commit_message>
<xml_diff>
--- a/docs/bd-news-sources.xlsx
+++ b/docs/bd-news-sources.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="299">
   <si>
     <t xml:space="preserve">Bangladeshi news portals — fetchability summary</t>
   </si>
@@ -165,6 +165,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://bangla.thedailystar.net/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/news-\d{5,}$</t>
   </si>
   <si>
     <t xml:space="preserve">/rss.xml stale (Feb 2026)</t>
@@ -1889,10 +1892,10 @@
       </c>
       <c r="H5" s="12"/>
       <c r="I5" s="15" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1900,29 +1903,29 @@
         <v>5</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F6" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H6" s="12"/>
       <c r="I6" s="15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1930,29 +1933,29 @@
         <v>6</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>5</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F7" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H7" s="12"/>
       <c r="I7" s="15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1960,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>5</v>
@@ -1969,20 +1972,20 @@
         <v>30</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F8" s="12" t="s">
         <v>9</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I8" s="15"/>
       <c r="J8" s="15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1990,29 +1993,29 @@
         <v>8</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F9" s="12" t="s">
         <v>9</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I9" s="15"/>
       <c r="J9" s="15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2020,7 +2023,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>5</v>
@@ -2029,20 +2032,20 @@
         <v>30</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F10" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H10" s="12"/>
       <c r="I10" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J10" s="15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2050,7 +2053,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>4</v>
@@ -2059,20 +2062,20 @@
         <v>30</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F11" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H11" s="12"/>
       <c r="I11" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J11" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2080,7 +2083,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C12" s="12" t="s">
         <v>4</v>
@@ -2089,20 +2092,20 @@
         <v>30</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F12" s="12" t="s">
         <v>9</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I12" s="15"/>
       <c r="J12" s="15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2110,7 +2113,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C13" s="12" t="s">
         <v>4</v>
@@ -2119,20 +2122,20 @@
         <v>30</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F13" s="12" t="s">
         <v>9</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I13" s="15"/>
       <c r="J13" s="15" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2140,7 +2143,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C14" s="12" t="s">
         <v>4</v>
@@ -2149,20 +2152,20 @@
         <v>30</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F14" s="12" t="s">
         <v>13</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I14" s="15"/>
       <c r="J14" s="15" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2170,7 +2173,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C15" s="12" t="s">
         <v>4</v>
@@ -2179,20 +2182,20 @@
         <v>30</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F15" s="12" t="s">
         <v>9</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I15" s="15"/>
       <c r="J15" s="15" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2200,7 +2203,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C16" s="12" t="s">
         <v>4</v>
@@ -2209,7 +2212,7 @@
         <v>30</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F16" s="12" t="s">
         <v>15</v>
@@ -2218,7 +2221,7 @@
       <c r="H16" s="12"/>
       <c r="I16" s="15"/>
       <c r="J16" s="15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2226,7 +2229,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>4</v>
@@ -2235,20 +2238,20 @@
         <v>30</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F17" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G17" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H17" s="12"/>
       <c r="I17" s="15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J17" s="15" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2256,7 +2259,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C18" s="12" t="s">
         <v>4</v>
@@ -2265,20 +2268,20 @@
         <v>30</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F18" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G18" s="14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H18" s="12"/>
       <c r="I18" s="15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J18" s="15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2286,7 +2289,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C19" s="12" t="s">
         <v>4</v>
@@ -2295,20 +2298,20 @@
         <v>30</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F19" s="12" t="s">
         <v>9</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I19" s="15"/>
       <c r="J19" s="15" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2316,7 +2319,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C20" s="12" t="s">
         <v>4</v>
@@ -2325,20 +2328,20 @@
         <v>30</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F20" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H20" s="12"/>
       <c r="I20" s="15" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J20" s="15" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2346,7 +2349,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C21" s="12" t="s">
         <v>4</v>
@@ -2355,16 +2358,16 @@
         <v>30</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F21" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G21" s="14" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I21" s="15"/>
       <c r="J21" s="15" t="s">
@@ -2376,7 +2379,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C22" s="12" t="s">
         <v>4</v>
@@ -2385,20 +2388,20 @@
         <v>30</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F22" s="12" t="s">
         <v>13</v>
       </c>
       <c r="G22" s="15" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I22" s="15"/>
       <c r="J22" s="15" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2406,7 +2409,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>4</v>
@@ -2415,7 +2418,7 @@
         <v>30</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F23" s="12" t="s">
         <v>15</v>
@@ -2424,7 +2427,7 @@
       <c r="H23" s="12"/>
       <c r="I23" s="15"/>
       <c r="J23" s="15" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2432,7 +2435,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C24" s="12" t="s">
         <v>4</v>
@@ -2441,7 +2444,7 @@
         <v>30</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F24" s="12" t="s">
         <v>15</v>
@@ -2450,7 +2453,7 @@
       <c r="H24" s="12"/>
       <c r="I24" s="15"/>
       <c r="J24" s="15" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2458,7 +2461,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C25" s="12" t="s">
         <v>4</v>
@@ -2467,20 +2470,20 @@
         <v>30</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F25" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G25" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H25" s="12"/>
       <c r="I25" s="15" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J25" s="15" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2488,7 +2491,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C26" s="12" t="s">
         <v>4</v>
@@ -2497,7 +2500,7 @@
         <v>30</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F26" s="12" t="s">
         <v>15</v>
@@ -2506,7 +2509,7 @@
       <c r="H26" s="12"/>
       <c r="I26" s="15"/>
       <c r="J26" s="15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2514,7 +2517,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C27" s="12" t="s">
         <v>4</v>
@@ -2523,20 +2526,20 @@
         <v>30</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F27" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G27" s="14" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H27" s="12" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I27" s="15"/>
       <c r="J27" s="15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2544,29 +2547,29 @@
         <v>27</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C28" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F28" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H28" s="12"/>
       <c r="I28" s="15" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J28" s="15" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2574,25 +2577,25 @@
         <v>28</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C29" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F29" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G29" s="14" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H29" s="12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I29" s="15"/>
       <c r="J29" s="15" t="s">
@@ -2604,25 +2607,25 @@
         <v>29</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C30" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F30" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G30" s="14" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I30" s="15"/>
       <c r="J30" s="15" t="s">
@@ -2634,16 +2637,16 @@
         <v>30</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C31" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F31" s="12" t="s">
         <v>15</v>
@@ -2652,7 +2655,7 @@
       <c r="H31" s="12"/>
       <c r="I31" s="15"/>
       <c r="J31" s="15" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2660,29 +2663,29 @@
         <v>31</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C32" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F32" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G32" s="14" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I32" s="15"/>
       <c r="J32" s="15" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2690,25 +2693,25 @@
         <v>32</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C33" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F33" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G33" s="14" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H33" s="12" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I33" s="15"/>
       <c r="J33" s="15" t="s">
@@ -2720,29 +2723,29 @@
         <v>33</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C34" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F34" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I34" s="15"/>
       <c r="J34" s="15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2750,29 +2753,29 @@
         <v>34</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C35" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F35" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G35" s="14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H35" s="12"/>
       <c r="I35" s="15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J35" s="15" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2780,16 +2783,16 @@
         <v>35</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C36" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F36" s="12" t="s">
         <v>15</v>
@@ -2798,7 +2801,7 @@
       <c r="H36" s="12"/>
       <c r="I36" s="15"/>
       <c r="J36" s="15" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2806,25 +2809,25 @@
         <v>36</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C37" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F37" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G37" s="14" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H37" s="12" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I37" s="15"/>
       <c r="J37" s="15" t="s">
@@ -2836,16 +2839,16 @@
         <v>37</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C38" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F38" s="12" t="s">
         <v>15</v>
@@ -2854,7 +2857,7 @@
       <c r="H38" s="12"/>
       <c r="I38" s="15"/>
       <c r="J38" s="15" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2862,29 +2865,29 @@
         <v>38</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C39" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E39" s="13" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F39" s="12" t="s">
         <v>9</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I39" s="15"/>
       <c r="J39" s="15" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2892,29 +2895,29 @@
         <v>39</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C40" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F40" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="H40" s="12" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I40" s="15"/>
       <c r="J40" s="15" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2922,29 +2925,29 @@
         <v>40</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C41" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F41" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G41" s="14" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H41" s="12"/>
       <c r="I41" s="15" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="J41" s="15" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2952,29 +2955,29 @@
         <v>41</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C42" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F42" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="H42" s="12"/>
       <c r="I42" s="15" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J42" s="15" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2982,29 +2985,29 @@
         <v>42</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C43" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F43" s="12" t="s">
         <v>9</v>
       </c>
       <c r="G43" s="14" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I43" s="15"/>
       <c r="J43" s="15" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3012,29 +3015,29 @@
         <v>43</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C44" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D44" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F44" s="12" t="s">
         <v>9</v>
       </c>
       <c r="G44" s="14" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H44" s="12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I44" s="15"/>
       <c r="J44" s="15" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3042,29 +3045,29 @@
         <v>44</v>
       </c>
       <c r="B45" s="12" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C45" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F45" s="12" t="s">
         <v>9</v>
       </c>
       <c r="G45" s="14" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H45" s="12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I45" s="15"/>
       <c r="J45" s="15" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3072,16 +3075,16 @@
         <v>45</v>
       </c>
       <c r="B46" s="12" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C46" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F46" s="12" t="s">
         <v>15</v>
@@ -3090,7 +3093,7 @@
       <c r="H46" s="12"/>
       <c r="I46" s="15"/>
       <c r="J46" s="15" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3098,29 +3101,29 @@
         <v>46</v>
       </c>
       <c r="B47" s="12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C47" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F47" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G47" s="14" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H47" s="12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I47" s="15"/>
       <c r="J47" s="15" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3128,7 +3131,7 @@
         <v>47</v>
       </c>
       <c r="B48" s="12" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C48" s="12" t="s">
         <v>4</v>
@@ -3137,20 +3140,20 @@
         <v>30</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F48" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G48" s="14" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H48" s="12"/>
       <c r="I48" s="15" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J48" s="15" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3158,7 +3161,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="12" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C49" s="12" t="s">
         <v>4</v>
@@ -3167,16 +3170,16 @@
         <v>30</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F49" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H49" s="12" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="I49" s="15"/>
       <c r="J49" s="15" t="s">
@@ -3188,7 +3191,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="12" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C50" s="12" t="s">
         <v>5</v>
@@ -3197,20 +3200,20 @@
         <v>30</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F50" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H50" s="12"/>
       <c r="I50" s="15" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="J50" s="15" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3218,7 +3221,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="12" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C51" s="12" t="s">
         <v>5</v>
@@ -3227,7 +3230,7 @@
         <v>30</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F51" s="12" t="s">
         <v>15</v>
@@ -3236,7 +3239,7 @@
       <c r="H51" s="12"/>
       <c r="I51" s="15"/>
       <c r="J51" s="15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3244,7 +3247,7 @@
         <v>51</v>
       </c>
       <c r="B52" s="12" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C52" s="12" t="s">
         <v>5</v>
@@ -3253,20 +3256,20 @@
         <v>30</v>
       </c>
       <c r="E52" s="13" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F52" s="12" t="s">
         <v>9</v>
       </c>
       <c r="G52" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="H52" s="12" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="I52" s="15"/>
       <c r="J52" s="15" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3274,7 +3277,7 @@
         <v>52</v>
       </c>
       <c r="B53" s="12" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C53" s="12" t="s">
         <v>5</v>
@@ -3283,20 +3286,20 @@
         <v>30</v>
       </c>
       <c r="E53" s="13" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F53" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G53" s="14" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="H53" s="12" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I53" s="15"/>
       <c r="J53" s="15" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3304,7 +3307,7 @@
         <v>53</v>
       </c>
       <c r="B54" s="12" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C54" s="12" t="s">
         <v>5</v>
@@ -3313,7 +3316,7 @@
         <v>30</v>
       </c>
       <c r="E54" s="13" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F54" s="12" t="s">
         <v>15</v>
@@ -3322,7 +3325,7 @@
       <c r="H54" s="12"/>
       <c r="I54" s="15"/>
       <c r="J54" s="15" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3330,7 +3333,7 @@
         <v>54</v>
       </c>
       <c r="B55" s="12" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C55" s="12" t="s">
         <v>5</v>
@@ -3339,20 +3342,20 @@
         <v>30</v>
       </c>
       <c r="E55" s="13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F55" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G55" s="14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="H55" s="12"/>
       <c r="I55" s="15" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J55" s="15" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3360,7 +3363,7 @@
         <v>55</v>
       </c>
       <c r="B56" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C56" s="12" t="s">
         <v>4</v>
@@ -3369,20 +3372,20 @@
         <v>30</v>
       </c>
       <c r="E56" s="13" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F56" s="12" t="s">
         <v>13</v>
       </c>
       <c r="G56" s="14" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="H56" s="12" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I56" s="15"/>
       <c r="J56" s="15" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3390,29 +3393,29 @@
         <v>56</v>
       </c>
       <c r="B57" s="12" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C57" s="12" t="s">
         <v>5</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E57" s="13" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F57" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G57" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="H57" s="12"/>
       <c r="I57" s="15" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J57" s="15" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3420,27 +3423,27 @@
         <v>57</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C58" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E58" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F58" s="12" t="s">
         <v>13</v>
       </c>
       <c r="G58" s="14" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="H58" s="12"/>
       <c r="I58" s="15"/>
       <c r="J58" s="15" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3448,29 +3451,29 @@
         <v>58</v>
       </c>
       <c r="B59" s="12" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C59" s="12" t="s">
         <v>5</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E59" s="13" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F59" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G59" s="14" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H59" s="12"/>
       <c r="I59" s="15" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J59" s="15" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3478,7 +3481,7 @@
         <v>59</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C60" s="12" t="s">
         <v>5</v>
@@ -3487,20 +3490,20 @@
         <v>30</v>
       </c>
       <c r="E60" s="13" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F60" s="12" t="s">
         <v>13</v>
       </c>
       <c r="G60" s="15" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H60" s="12" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="I60" s="15"/>
       <c r="J60" s="15" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3508,7 +3511,7 @@
         <v>60</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C61" s="12" t="s">
         <v>4</v>
@@ -3517,20 +3520,20 @@
         <v>30</v>
       </c>
       <c r="E61" s="13" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F61" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G61" s="14" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="H61" s="12"/>
       <c r="I61" s="15" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J61" s="15" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3538,7 +3541,7 @@
         <v>61</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C62" s="12" t="s">
         <v>4</v>
@@ -3547,20 +3550,20 @@
         <v>30</v>
       </c>
       <c r="E62" s="13" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F62" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G62" s="14" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="H62" s="12" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="I62" s="15"/>
       <c r="J62" s="15" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3568,7 +3571,7 @@
         <v>62</v>
       </c>
       <c r="B63" s="12" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C63" s="12" t="s">
         <v>4</v>
@@ -3577,7 +3580,7 @@
         <v>30</v>
       </c>
       <c r="E63" s="13" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F63" s="12" t="s">
         <v>15</v>
@@ -3586,7 +3589,7 @@
       <c r="H63" s="12"/>
       <c r="I63" s="15"/>
       <c r="J63" s="15" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3594,7 +3597,7 @@
         <v>63</v>
       </c>
       <c r="B64" s="12" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C64" s="12" t="s">
         <v>4</v>
@@ -3603,16 +3606,16 @@
         <v>30</v>
       </c>
       <c r="E64" s="13" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F64" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G64" s="14" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="H64" s="12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I64" s="15"/>
       <c r="J64" s="15" t="s">
@@ -3624,7 +3627,7 @@
         <v>64</v>
       </c>
       <c r="B65" s="12" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C65" s="12" t="s">
         <v>4</v>
@@ -3633,25 +3636,25 @@
         <v>30</v>
       </c>
       <c r="E65" s="13" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F65" s="12" t="s">
         <v>9</v>
       </c>
       <c r="G65" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="H65" s="12" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="I65" s="15"/>
       <c r="J65" s="15" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>